<commit_message>
added column renamer pointer for admie.IMBABE
</commit_message>
<xml_diff>
--- a/exso/Files/ReportsInfo.xlsx
+++ b/exso/Files/ReportsInfo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20827"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.natsikas\Desktop\Admie-Desktop\Projects\exso\exso\exso\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thanos\Desktop\Admie-Desktop\Projects\exso\exso\exso\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA4ACF1-EE57-4CCA-ACF0-5BE54D9362BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF703AC-3EC3-4CEA-80C2-544837132E58}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,19 +26,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Read Settings'!$A$1:$I$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Time Settings'!$A$1:$J$120</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="179021"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -1209,7 +1198,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="342">
   <si>
     <t>Report Name</t>
   </si>
@@ -2233,6 +2222,12 @@
   </si>
   <si>
     <t>{'FYROM':'NORTH MACEDONIA', 'CET Hour': 'Hour (CET)'}</t>
+  </si>
+  <si>
+    <t>{'ΝΕΤ CBS SCHEDULES': 'NET CBS SCHEDULES'}</t>
+  </si>
+  <si>
+    <t>IMBABE.csv</t>
   </si>
 </sst>
 </file>
@@ -3680,9 +3675,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3720,7 +3715,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3826,7 +3821,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3968,7 +3963,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -10657,7 +10652,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L120" xr:uid="{D0972C50-907B-4A2C-82F0-ED51F06329AA}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L120">
+    <sortState ref="A2:L120">
       <sortCondition ref="A2:A120"/>
     </sortState>
   </autoFilter>
@@ -15684,7 +15679,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I111" xr:uid="{776C4DE2-2957-440A-A09D-B0AB3152981D}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I120">
+    <sortState ref="A2:I120">
       <sortCondition ref="A1:A111"/>
     </sortState>
   </autoFilter>
@@ -15980,7 +15975,9 @@
       </c>
       <c r="D11" s="24"/>
       <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>340</v>
+      </c>
       <c r="G11" s="12" t="s">
         <v>246</v>
       </c>
@@ -17278,7 +17275,9 @@
         <v>1</v>
       </c>
       <c r="C70" s="23"/>
-      <c r="D70" s="24"/>
+      <c r="D70" s="24" t="s">
+        <v>341</v>
+      </c>
       <c r="E70" s="23"/>
       <c r="F70" s="8"/>
       <c r="G70" s="12" t="s">
@@ -20203,7 +20202,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I109" xr:uid="{44BD8FFD-EDA1-47AD-AC03-3890015323F4}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I120">
+    <sortState ref="A2:I120">
       <sortCondition ref="A1:A109"/>
     </sortState>
   </autoFilter>
@@ -26798,7 +26797,7 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="37">
         <f ca="1">NOW()</f>
-        <v>45967.468476851849</v>
+        <v>46134.461413425925</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>